<commit_message>
update press speed and dashboard
</commit_message>
<xml_diff>
--- a/Generator/simulation_inputs.xlsx
+++ b/Generator/simulation_inputs.xlsx
@@ -8,33 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rr441707/Documents/Wil/Python/Project/Generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1101562E-FAF2-D747-A357-35AE8275137A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05A0AB66-57F5-234B-B9AF-6FC3007D6EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main Control Panel" sheetId="1" r:id="rId1"/>
     <sheet name="Backend Engine" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="158">
   <si>
     <t>1. Scenario Metadata</t>
   </si>
@@ -225,13 +212,19 @@
     <t>SHEETFED_RATE_HR</t>
   </si>
   <si>
-    <t>Actual cost to run SF press per hour (fully loaded)</t>
+    <t>Actual cost to run SF press per hour (direct labor only)</t>
   </si>
   <si>
     <t>PERFECTING_RATE_HR</t>
   </si>
   <si>
-    <t>Actual cost to run PF press per hour (fully loaded)</t>
+    <t>Actual cost to run PF press per hour (direct labor only)</t>
+  </si>
+  <si>
+    <t>BURDEN_RATE_HR</t>
+  </si>
+  <si>
+    <t>Overhead allocation per press hour — add when known (rent, utilities, depreciation)</t>
   </si>
   <si>
     <t>SHEETFED_BILL_RATE_HR</t>
@@ -262,6 +255,12 @@
   </si>
   <si>
     <t>Cost of ink per lb</t>
+  </si>
+  <si>
+    <t>INK_YIELD_SHEETS_PER_LB</t>
+  </si>
+  <si>
+    <t>Sheet-sides per lb of ink at 100% coverage — calibrate against real consumption data</t>
   </si>
   <si>
     <t>3. Base Speeds &amp; Output Math</t>
@@ -1145,7 +1144,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1260,7 +1259,7 @@
         <v>66</v>
       </c>
       <c r="B12">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="C12" t="s">
         <v>67</v>
@@ -1271,7 +1270,7 @@
         <v>68</v>
       </c>
       <c r="B13">
-        <v>285</v>
+        <v>250</v>
       </c>
       <c r="C13" t="s">
         <v>69</v>
@@ -1282,7 +1281,7 @@
         <v>70</v>
       </c>
       <c r="B14">
-        <v>55</v>
+        <v>285</v>
       </c>
       <c r="C14" t="s">
         <v>71</v>
@@ -1293,7 +1292,7 @@
         <v>72</v>
       </c>
       <c r="B15">
-        <v>320</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
         <v>73</v>
@@ -1304,47 +1303,47 @@
         <v>74</v>
       </c>
       <c r="B16">
-        <v>20</v>
+        <v>320</v>
       </c>
       <c r="C16" t="s">
         <v>75</v>
       </c>
     </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>77</v>
+      </c>
+    </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B19">
-        <v>0.8</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="A18" s="1" t="s">
         <v>78</v>
       </c>
+      <c r="B18">
+        <v>50000</v>
+      </c>
+      <c r="C18" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B20">
-        <v>10500</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="A20" s="2" t="s">
         <v>80</v>
       </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B21">
-        <v>9500</v>
+        <v>0.8</v>
       </c>
       <c r="C21" t="s">
         <v>82</v>
@@ -1355,7 +1354,7 @@
         <v>83</v>
       </c>
       <c r="B22">
-        <v>7500</v>
+        <v>10500</v>
       </c>
       <c r="C22" t="s">
         <v>84</v>
@@ -1366,47 +1365,47 @@
         <v>85</v>
       </c>
       <c r="B23">
-        <v>6500</v>
+        <v>9500</v>
       </c>
       <c r="C23" t="s">
         <v>86</v>
       </c>
     </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24">
+        <v>7500</v>
+      </c>
+      <c r="C24" t="s">
+        <v>88</v>
+      </c>
+    </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B26">
-        <v>3.5</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="A25" s="1" t="s">
         <v>89</v>
       </c>
+      <c r="B25">
+        <v>6500</v>
+      </c>
+      <c r="C25" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B27">
-        <v>2</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="A27" s="2" t="s">
         <v>91</v>
       </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B28">
-        <v>30</v>
+        <v>3.5</v>
       </c>
       <c r="C28" t="s">
         <v>93</v>
@@ -1417,7 +1416,7 @@
         <v>94</v>
       </c>
       <c r="B29">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="C29" t="s">
         <v>95</v>
@@ -1428,47 +1427,47 @@
         <v>96</v>
       </c>
       <c r="B30">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="C30" t="s">
         <v>97</v>
       </c>
     </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B31">
+        <v>0.5</v>
+      </c>
+      <c r="C31" t="s">
+        <v>99</v>
+      </c>
+    </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B33">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="A32" s="1" t="s">
         <v>100</v>
       </c>
+      <c r="B32">
+        <v>70</v>
+      </c>
+      <c r="C32" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B34">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="A34" s="2" t="s">
         <v>102</v>
       </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>103</v>
       </c>
       <c r="B35">
-        <v>1.25</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="C35" t="s">
         <v>104</v>
@@ -1479,7 +1478,7 @@
         <v>105</v>
       </c>
       <c r="B36">
-        <v>400</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="C36" t="s">
         <v>106</v>
@@ -1490,7 +1489,7 @@
         <v>107</v>
       </c>
       <c r="B37">
-        <v>0.55000000000000004</v>
+        <v>1.25</v>
       </c>
       <c r="C37" t="s">
         <v>108</v>
@@ -1501,7 +1500,7 @@
         <v>109</v>
       </c>
       <c r="B38">
-        <v>0.9</v>
+        <v>400</v>
       </c>
       <c r="C38" t="s">
         <v>110</v>
@@ -1512,7 +1511,7 @@
         <v>111</v>
       </c>
       <c r="B39">
-        <v>50</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="C39" t="s">
         <v>112</v>
@@ -1523,7 +1522,7 @@
         <v>113</v>
       </c>
       <c r="B40">
-        <v>15</v>
+        <v>0.9</v>
       </c>
       <c r="C40" t="s">
         <v>114</v>
@@ -1534,87 +1533,87 @@
         <v>115</v>
       </c>
       <c r="B41">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="C41" t="s">
         <v>116</v>
       </c>
     </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B42">
+        <v>15</v>
+      </c>
+      <c r="C42" t="s">
+        <v>118</v>
+      </c>
+    </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B44">
-        <v>0.03</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="A43" s="1" t="s">
         <v>119</v>
       </c>
+      <c r="B43">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="B45">
-        <v>20</v>
-      </c>
-      <c r="C45" t="s">
+      <c r="A45" s="2" t="s">
         <v>121</v>
       </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>122</v>
       </c>
       <c r="B46">
-        <v>30</v>
+        <v>0.03</v>
       </c>
       <c r="C46" t="s">
         <v>123</v>
       </c>
     </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B47">
+        <v>20</v>
+      </c>
+      <c r="C47" t="s">
+        <v>125</v>
+      </c>
+    </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B49">
-        <v>7</v>
-      </c>
-      <c r="C49" t="s">
+      <c r="A48" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="B48">
+        <v>30</v>
+      </c>
+      <c r="C48" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B50">
-        <v>2</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="A50" s="2" t="s">
         <v>128</v>
       </c>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>129</v>
       </c>
       <c r="B51">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C51" t="s">
         <v>130</v>
@@ -1625,7 +1624,7 @@
         <v>131</v>
       </c>
       <c r="B52">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C52" t="s">
         <v>132</v>
@@ -1636,47 +1635,47 @@
         <v>133</v>
       </c>
       <c r="B53">
-        <v>0.75</v>
+        <v>6</v>
       </c>
       <c r="C53" t="s">
         <v>134</v>
       </c>
     </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B54">
+        <v>24</v>
+      </c>
+      <c r="C54" t="s">
+        <v>136</v>
+      </c>
+    </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B56">
-        <v>0.7</v>
-      </c>
-      <c r="C56" t="s">
+      <c r="A55" s="1" t="s">
         <v>137</v>
       </c>
+      <c r="B55">
+        <v>0.75</v>
+      </c>
+      <c r="C55" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B57">
-        <v>0.2</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="A57" s="2" t="s">
         <v>139</v>
       </c>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B58">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="C58" t="s">
         <v>141</v>
@@ -1687,47 +1686,47 @@
         <v>142</v>
       </c>
       <c r="B59">
-        <v>42</v>
+        <v>0.2</v>
       </c>
       <c r="C59" t="s">
         <v>143</v>
       </c>
     </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B60">
+        <v>0.1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>145</v>
+      </c>
+    </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B61" s="3"/>
-      <c r="C61" s="3"/>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="B62" t="s">
+      <c r="A61" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C62" t="s">
+      <c r="B61">
+        <v>42</v>
+      </c>
+      <c r="C61" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="1" t="s">
+      <c r="A63" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B63" t="s">
-        <v>146</v>
-      </c>
-      <c r="C63" t="s">
-        <v>149</v>
-      </c>
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B64" t="s">
         <v>150</v>
-      </c>
-      <c r="B64" t="s">
-        <v>146</v>
       </c>
       <c r="C64" t="s">
         <v>151</v>
@@ -1738,23 +1737,45 @@
         <v>152</v>
       </c>
       <c r="B65" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C65" t="s">
         <v>153</v>
       </c>
     </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B66" t="s">
+        <v>150</v>
+      </c>
+      <c r="C66" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B67" t="s">
+        <v>150</v>
+      </c>
+      <c r="C67" t="s">
+        <v>157</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A63:C63"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A57:C57"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A20:C20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>